<commit_message>
fix production allowed host handling
</commit_message>
<xml_diff>
--- a/docs/BUG_TRACKER.xlsx
+++ b/docs/BUG_TRACKER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\source\repos\DailyVitalsApp\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2788C3E7-4D91-420F-A4F2-906274E9DAA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D60F2AAE-2A82-4C33-BB75-E1DCC9E053FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="185">
   <si>
     <t>Bug ID</t>
   </si>
@@ -578,6 +578,21 @@
   </si>
   <si>
     <t>The details modal pop message should show values</t>
+  </si>
+  <si>
+    <t>feature/blood-pressure-save</t>
+  </si>
+  <si>
+    <t>SSR form-post binding failure</t>
+  </si>
+  <si>
+    <t>page isn't working message</t>
+  </si>
+  <si>
+    <t>page comes back with page isn't working</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-011.png</t>
   </si>
 </sst>
 </file>
@@ -1244,7 +1259,9 @@
       <c r="I5" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="J5" s="2"/>
+      <c r="J5" s="2" t="s">
+        <v>180</v>
+      </c>
       <c r="K5" s="2" t="s">
         <v>32</v>
       </c>
@@ -1254,7 +1271,9 @@
       <c r="M5" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="N5" s="2"/>
+      <c r="N5" t="s">
+        <v>181</v>
+      </c>
       <c r="O5" s="2"/>
       <c r="P5" s="2" t="s">
         <v>30</v>
@@ -1553,19 +1572,33 @@
       <c r="A12" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+      <c r="B12" s="3">
+        <v>46216</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>183</v>
+      </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="L12" s="2"/>
+      <c r="L12" s="2" t="s">
+        <v>184</v>
+      </c>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -1573,9 +1606,9 @@
         <v>30</v>
       </c>
       <c r="Q12" s="3"/>
-      <c r="R12" s="4" t="str">
+      <c r="R12" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:18">
@@ -2212,7 +2245,7 @@
       </c>
       <c r="Q34" s="3"/>
       <c r="R34" s="4" t="str">
-        <f t="shared" ref="R34:R65" ca="1" si="1">IF(B34="","",IF(Q34&lt;&gt;"",Q34-B34,TODAY()-B34))</f>
+        <f t="shared" ref="R34:R51" ca="1" si="1">IF(B34="","",IF(Q34&lt;&gt;"",Q34-B34,TODAY()-B34))</f>
         <v/>
       </c>
     </row>
@@ -2829,7 +2862,7 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIF('Bug Tracker'!F2:F51,"&lt;&gt;")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5" t="s">
@@ -2845,7 +2878,7 @@
       </c>
       <c r="H5" s="5">
         <f>COUNTIF('Bug Tracker'!C2:C51,G5)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2854,7 +2887,7 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIFS('Bug Tracker'!F2:F51,"&lt;&gt;",'Bug Tracker'!K2:K51,"&lt;&gt;Closed",'Bug Tracker'!K2:K51,"&lt;&gt;Verified")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
@@ -2879,7 +2912,7 @@
       </c>
       <c r="B7" s="5">
         <f>COUNTIF('Bug Tracker'!C2:C51,"Critical")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">

</xml_diff>

<commit_message>
update bug tracker and screenshots
</commit_message>
<xml_diff>
--- a/docs/BUG_TRACKER.xlsx
+++ b/docs/BUG_TRACKER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\source\repos\DailyVitalsApp\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36F14DCB-38B7-4CF1-AC7B-9BEA569C8F7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD50265C-C818-4EF4-8C9D-E4E03FBBFBA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="252">
   <si>
     <t>Bug ID</t>
   </si>
@@ -715,6 +715,149 @@
   </si>
   <si>
     <t>kidney lab pop</t>
+  </si>
+  <si>
+    <t>time of entry is not default setting to CST, is this a setting in profile and then it will be according to the user local</t>
+  </si>
+  <si>
+    <t>Data Issue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CST time value </t>
+  </si>
+  <si>
+    <t>should be CST</t>
+  </si>
+  <si>
+    <t>appears east coat</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-017.png</t>
+  </si>
+  <si>
+    <t>hide Renal Friendly Foods menu for now</t>
+  </si>
+  <si>
+    <t>Enhancement</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>needs to be restructured to global foods not person specific</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-018.png</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-019.png</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-020.png</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-021.png</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-022.png</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-023.png</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-024.png</t>
+  </si>
+  <si>
+    <t>plain server POST endpoint</t>
+  </si>
+  <si>
+    <t>feature/add-new-exercise</t>
+  </si>
+  <si>
+    <t>35d218d</t>
+  </si>
+  <si>
+    <t>delete button remains disabled for selected item, it should be able to delete as normal</t>
+  </si>
+  <si>
+    <t>delete button disabled</t>
+  </si>
+  <si>
+    <t>make selection and delete work through normal browser/server requests</t>
+  </si>
+  <si>
+    <t>932b0c2</t>
+  </si>
+  <si>
+    <t>feature/exercise-delete-button-disabled</t>
+  </si>
+  <si>
+    <t>move the save action out of Blazor validation and into a server endpoint</t>
+  </si>
+  <si>
+    <t>66b11c5</t>
+  </si>
+  <si>
+    <t>fluid intake delete</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">verify the menu no longer has those fragile </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>@onclick</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Carlito"/>
+      </rPr>
+      <t xml:space="preserve"> submenu buttons</t>
+    </r>
+  </si>
+  <si>
+    <t>feature/nutrition-sub-menu-load-failure</t>
+  </si>
+  <si>
+    <t>fa23273</t>
+  </si>
+  <si>
+    <t>add food item on save blanks fields out does nothing</t>
+  </si>
+  <si>
+    <t>nutrition save error</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">the modal exists, but the Details buttons are </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>@onclick</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Carlito"/>
+      </rPr>
+      <t xml:space="preserve"> only</t>
+    </r>
+  </si>
+  <si>
+    <t>d4b5ee6</t>
+  </si>
+  <si>
+    <t>8cfb9c4</t>
+  </si>
+  <si>
+    <t>remove delete button</t>
   </si>
 </sst>
 </file>
@@ -949,7 +1092,6 @@
   <autoFilter ref="A1:R51" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}">
     <filterColumn colId="10">
       <filters>
-        <filter val="Investigating"/>
         <filter val="Open"/>
       </filters>
     </filterColumn>
@@ -1153,7 +1295,7 @@
     <col min="6" max="6" width="28" customWidth="1"/>
     <col min="7" max="7" width="38" customWidth="1"/>
     <col min="8" max="9" width="32" customWidth="1"/>
-    <col min="10" max="10" width="27" customWidth="1"/>
+    <col min="10" max="10" width="33" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18" customWidth="1"/>
     <col min="12" max="12" width="30" customWidth="1"/>
     <col min="13" max="13" width="34" customWidth="1"/>
@@ -1220,7 +1362,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="42">
+    <row r="2" spans="1:18" ht="42" hidden="1">
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
@@ -1252,7 +1394,7 @@
         <v>26</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>27</v>
+        <v>95</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>28</v>
@@ -1268,7 +1410,7 @@
       <c r="Q2" s="3"/>
       <c r="R2" s="4">
         <f t="shared" ref="R2:R33" ca="1" si="0">IF(B2="","",IF(Q2&lt;&gt;"",Q2-B2,TODAY()-B2))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="28">
@@ -1315,7 +1457,7 @@
       <c r="Q3" s="3"/>
       <c r="R3" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:18" ht="28">
@@ -1362,7 +1504,7 @@
       <c r="Q4" s="3"/>
       <c r="R4" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="28" hidden="1">
@@ -1415,7 +1557,7 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="28" hidden="1">
@@ -1466,7 +1608,7 @@
       <c r="Q6" s="3"/>
       <c r="R6" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="28" hidden="1">
@@ -1570,7 +1712,7 @@
       <c r="Q8" s="3"/>
       <c r="R8" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="42" hidden="1">
@@ -1626,7 +1768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="28">
+    <row r="10" spans="1:18" ht="28" hidden="1">
       <c r="A10" s="2" t="s">
         <v>39</v>
       </c>
@@ -1654,26 +1796,32 @@
       <c r="I10" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="J10" s="2"/>
+      <c r="J10" s="2" t="s">
+        <v>233</v>
+      </c>
       <c r="K10" s="2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>164</v>
       </c>
       <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
+      <c r="N10" t="s">
+        <v>232</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>234</v>
+      </c>
       <c r="P10" s="2" t="s">
-        <v>30</v>
+        <v>186</v>
       </c>
       <c r="Q10" s="3"/>
       <c r="R10" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" ht="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="28" hidden="1">
       <c r="A11" s="2" t="s">
         <v>40</v>
       </c>
@@ -1703,21 +1851,27 @@
       </c>
       <c r="J11" s="2"/>
       <c r="K11" s="2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>165</v>
       </c>
       <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
+      <c r="N11" t="s">
+        <v>248</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>249</v>
+      </c>
       <c r="P11" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q11" s="3"/>
+        <v>186</v>
+      </c>
+      <c r="Q11" s="3">
+        <v>46217</v>
+      </c>
       <c r="R11" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:18" hidden="1">
@@ -1820,7 +1974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="28">
+    <row r="14" spans="1:18" ht="28" hidden="1">
       <c r="A14" s="2" t="s">
         <v>43</v>
       </c>
@@ -1850,22 +2004,28 @@
       </c>
       <c r="J14" s="2"/>
       <c r="K14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L14" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>230</v>
+      </c>
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
+      <c r="O14" s="2" t="s">
+        <v>250</v>
+      </c>
       <c r="P14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q14" s="3"/>
+        <v>186</v>
+      </c>
+      <c r="Q14" s="3">
+        <v>46217</v>
+      </c>
       <c r="R14" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" hidden="1">
       <c r="A15" s="2" t="s">
         <v>44</v>
       </c>
@@ -1891,26 +2051,34 @@
       <c r="I15" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="J15" s="2"/>
+      <c r="J15" s="2" t="s">
+        <v>244</v>
+      </c>
       <c r="K15" s="2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>205</v>
       </c>
       <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
+      <c r="N15" t="s">
+        <v>243</v>
+      </c>
+      <c r="O15" t="s">
+        <v>245</v>
+      </c>
       <c r="P15" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q15" s="3"/>
+        <v>186</v>
+      </c>
+      <c r="Q15" s="3">
+        <v>46217</v>
+      </c>
       <c r="R15" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18" ht="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="28" hidden="1">
       <c r="A16" s="2" t="s">
         <v>45</v>
       </c>
@@ -1936,21 +2104,27 @@
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L16" s="2" t="s">
         <v>209</v>
       </c>
       <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
+      <c r="N16" t="s">
+        <v>240</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>241</v>
+      </c>
       <c r="P16" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q16" s="3"/>
+        <v>186</v>
+      </c>
+      <c r="Q16" s="3">
+        <v>46217</v>
+      </c>
       <c r="R16" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="28">
@@ -1993,7 +2167,7 @@
       <c r="Q17" s="3"/>
       <c r="R17" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:18" ht="28">
@@ -2026,7 +2200,9 @@
       <c r="K18" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="L18" s="2"/>
+      <c r="L18" s="2" t="s">
+        <v>220</v>
+      </c>
       <c r="M18" s="2"/>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -2036,26 +2212,44 @@
       <c r="Q18" s="3"/>
       <c r="R18" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="42">
       <c r="A19" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
+      <c r="B19" s="3">
+        <v>46217</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>219</v>
+      </c>
       <c r="J19" s="2"/>
       <c r="K19" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="L19" s="2"/>
+      <c r="L19" s="2" t="s">
+        <v>225</v>
+      </c>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -2063,28 +2257,42 @@
         <v>30</v>
       </c>
       <c r="Q19" s="3"/>
-      <c r="R19" s="4" t="str">
+      <c r="R19" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="1:18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="28">
       <c r="A20" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
+      <c r="B20" s="3">
+        <v>46217</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>224</v>
+      </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="L20" s="2"/>
+      <c r="L20" s="2" t="s">
+        <v>226</v>
+      </c>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -2092,57 +2300,93 @@
         <v>30</v>
       </c>
       <c r="Q20" s="3"/>
-      <c r="R20" s="4" t="str">
+      <c r="R20" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="1:18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="28" hidden="1">
       <c r="A21" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="B21" s="3">
+        <v>46217</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>235</v>
+      </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
+      <c r="J21" s="2" t="s">
+        <v>239</v>
+      </c>
       <c r="K21" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L21" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>227</v>
+      </c>
       <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
+      <c r="N21" t="s">
+        <v>237</v>
+      </c>
+      <c r="O21" s="2" t="s">
+        <v>238</v>
+      </c>
       <c r="P21" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q21" s="3"/>
-      <c r="R21" s="4" t="str">
+        <v>186</v>
+      </c>
+      <c r="Q21" s="3">
+        <v>46217</v>
+      </c>
+      <c r="R21" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" ht="28">
       <c r="A22" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
+      <c r="B22" s="3">
+        <v>46217</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>235</v>
+      </c>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="L22" s="2"/>
+      <c r="L22" s="2" t="s">
+        <v>228</v>
+      </c>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -2150,28 +2394,42 @@
         <v>30</v>
       </c>
       <c r="Q22" s="3"/>
-      <c r="R22" s="4" t="str">
+      <c r="R22" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" ht="28">
       <c r="A23" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="2"/>
-      <c r="G23" s="2"/>
+      <c r="B23" s="3">
+        <v>46217</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>246</v>
+      </c>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="L23" s="2"/>
+      <c r="L23" s="2" t="s">
+        <v>229</v>
+      </c>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -2179,20 +2437,30 @@
         <v>30</v>
       </c>
       <c r="Q23" s="3"/>
-      <c r="R23" s="4" t="str">
+      <c r="R23" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:18">
       <c r="A24" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B24" s="3"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
+      <c r="B24" s="3">
+        <v>46217</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>251</v>
+      </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
@@ -2200,7 +2468,9 @@
       <c r="K24" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="L24" s="2"/>
+      <c r="L24" s="2" t="s">
+        <v>231</v>
+      </c>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -2208,9 +2478,9 @@
         <v>30</v>
       </c>
       <c r="Q24" s="3"/>
-      <c r="R24" s="4" t="str">
+      <c r="R24" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:18">
@@ -3047,8 +3317,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -3116,7 +3387,7 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIF('Bug Tracker'!F2:F51,"&lt;&gt;")</f>
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5" t="s">
@@ -3124,7 +3395,7 @@
       </c>
       <c r="E5" s="5">
         <f>COUNTIF('Bug Tracker'!K2:K51,D5)</f>
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="F5" s="5"/>
       <c r="G5" s="5" t="s">
@@ -3132,7 +3403,7 @@
       </c>
       <c r="H5" s="5">
         <f>COUNTIF('Bug Tracker'!C2:C51,G5)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -3141,7 +3412,7 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIFS('Bug Tracker'!F2:F51,"&lt;&gt;",'Bug Tracker'!K2:K51,"&lt;&gt;Closed",'Bug Tracker'!K2:K51,"&lt;&gt;Verified")</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
@@ -3149,7 +3420,7 @@
       </c>
       <c r="E6" s="5">
         <f>COUNTIF('Bug Tracker'!K2:K51,D6)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5" t="s">
@@ -3157,7 +3428,7 @@
       </c>
       <c r="H6" s="5">
         <f>COUNTIF('Bug Tracker'!C2:C51,G6)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -3166,7 +3437,7 @@
       </c>
       <c r="B7" s="5">
         <f>COUNTIF('Bug Tracker'!C2:C51,"Critical")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
@@ -3191,7 +3462,7 @@
       </c>
       <c r="B8" s="5">
         <f>COUNTIF('Bug Tracker'!C2:C51,"High")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5" t="s">
@@ -3207,7 +3478,7 @@
       </c>
       <c r="H8" s="5">
         <f>COUNTIF('Bug Tracker'!C2:C51,G8)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -3256,7 +3527,7 @@
       </c>
       <c r="B11" s="5">
         <f>COUNTIF('Bug Tracker'!K2:K51,"Closed")+COUNTIF('Bug Tracker'!K2:K51,"Verified")</f>
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5" t="s">
@@ -3294,7 +3565,7 @@
       </c>
       <c r="E13" s="5">
         <f>COUNTIF('Bug Tracker'!K2:K51,D13)</f>
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>

</xml_diff>

<commit_message>
bug tracker and screenshots update
</commit_message>
<xml_diff>
--- a/docs/BUG_TRACKER.xlsx
+++ b/docs/BUG_TRACKER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\source\repos\DailyVitalsApp\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD50265C-C818-4EF4-8C9D-E4E03FBBFBA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D07055B-BE61-40C9-A9A7-9B89ECB2AA90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="272">
   <si>
     <t>Bug ID</t>
   </si>
@@ -858,6 +858,66 @@
   </si>
   <si>
     <t>remove delete button</t>
+  </si>
+  <si>
+    <t>time change should automatically update the Notes as shown, does nothing</t>
+  </si>
+  <si>
+    <t>update time</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-025.png</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-026.png</t>
+  </si>
+  <si>
+    <t>delete button is remains disabled, user should be able to change fluid records</t>
+  </si>
+  <si>
+    <t>disable delete button</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-027.png</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-028.png</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-030.png</t>
+  </si>
+  <si>
+    <t>docs/screenshots/AV-031.png</t>
+  </si>
+  <si>
+    <t>all buttons New, Delete and Save are inoperable</t>
+  </si>
+  <si>
+    <t>inoperable buttons</t>
+  </si>
+  <si>
+    <t>23f1cbe</t>
+  </si>
+  <si>
+    <t>New button should reset the page and clear the validation errors but does nothing</t>
+  </si>
+  <si>
+    <t>New button inoperable</t>
+  </si>
+  <si>
+    <t>Save blanks out form and does not save newly entered food item</t>
+  </si>
+  <si>
+    <t>Save new food inoperable</t>
+  </si>
+  <si>
+    <t>interactive server connection is falling back to a normal POST</t>
+  </si>
+  <si>
+    <t>feature/inoperable-save-new-food-button</t>
+  </si>
+  <si>
+    <t>56abd35  58ecfef  3ba3a1c</t>
   </si>
 </sst>
 </file>
@@ -1410,7 +1470,7 @@
       <c r="Q2" s="3"/>
       <c r="R2" s="4">
         <f t="shared" ref="R2:R33" ca="1" si="0">IF(B2="","",IF(Q2&lt;&gt;"",Q2-B2,TODAY()-B2))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="28">
@@ -1443,7 +1503,7 @@
       </c>
       <c r="J3" s="2"/>
       <c r="K3" s="2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>137</v>
@@ -1457,10 +1517,10 @@
       <c r="Q3" s="3"/>
       <c r="R3" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" ht="28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" ht="28" hidden="1">
       <c r="A4" s="2" t="s">
         <v>33</v>
       </c>
@@ -1490,7 +1550,7 @@
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>141</v>
@@ -1504,7 +1564,7 @@
       <c r="Q4" s="3"/>
       <c r="R4" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:18" ht="28" hidden="1">
@@ -1557,7 +1617,7 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:18" ht="28" hidden="1">
@@ -1608,7 +1668,7 @@
       <c r="Q6" s="3"/>
       <c r="R6" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="28" hidden="1">
@@ -1712,7 +1772,7 @@
       <c r="Q8" s="3"/>
       <c r="R8" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="42" hidden="1">
@@ -1818,7 +1878,7 @@
       <c r="Q10" s="3"/>
       <c r="R10" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="28" hidden="1">
@@ -2127,7 +2187,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="28">
+    <row r="17" spans="1:18" ht="28" hidden="1">
       <c r="A17" s="2" t="s">
         <v>46</v>
       </c>
@@ -2153,7 +2213,7 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>212</v>
@@ -2162,15 +2222,15 @@
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
       <c r="P17" s="2" t="s">
-        <v>30</v>
+        <v>186</v>
       </c>
       <c r="Q17" s="3"/>
       <c r="R17" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" ht="28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="28" hidden="1">
       <c r="A18" s="2" t="s">
         <v>47</v>
       </c>
@@ -2198,7 +2258,7 @@
       </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L18" s="2" t="s">
         <v>220</v>
@@ -2212,10 +2272,10 @@
       <c r="Q18" s="3"/>
       <c r="R18" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18" ht="42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="42" hidden="1">
       <c r="A19" s="2" t="s">
         <v>48</v>
       </c>
@@ -2245,7 +2305,7 @@
       </c>
       <c r="J19" s="2"/>
       <c r="K19" s="2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>225</v>
@@ -2259,10 +2319,10 @@
       <c r="Q19" s="3"/>
       <c r="R19" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:18" ht="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="28" hidden="1">
       <c r="A20" s="2" t="s">
         <v>49</v>
       </c>
@@ -2288,7 +2348,7 @@
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>226</v>
@@ -2302,7 +2362,7 @@
       <c r="Q20" s="3"/>
       <c r="R20" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:18" ht="28" hidden="1">
@@ -2356,7 +2416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="28">
+    <row r="22" spans="1:18" ht="28" hidden="1">
       <c r="A22" s="2" t="s">
         <v>51</v>
       </c>
@@ -2382,7 +2442,7 @@
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L22" s="2" t="s">
         <v>228</v>
@@ -2391,15 +2451,17 @@
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
       <c r="P22" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q22" s="3"/>
+        <v>186</v>
+      </c>
+      <c r="Q22" s="3">
+        <v>46218</v>
+      </c>
       <c r="R22" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:18" ht="28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" ht="28" hidden="1">
       <c r="A23" s="2" t="s">
         <v>52</v>
       </c>
@@ -2425,7 +2487,7 @@
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L23" s="2" t="s">
         <v>229</v>
@@ -2434,15 +2496,17 @@
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
       <c r="P23" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q23" s="3"/>
+        <v>186</v>
+      </c>
+      <c r="Q23" s="3">
+        <v>46218</v>
+      </c>
       <c r="R23" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" hidden="1">
       <c r="A24" s="2" t="s">
         <v>53</v>
       </c>
@@ -2466,7 +2530,7 @@
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="L24" s="2" t="s">
         <v>231</v>
@@ -2480,26 +2544,40 @@
       <c r="Q24" s="3"/>
       <c r="R24" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" ht="28" hidden="1">
       <c r="A25" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="2"/>
+      <c r="B25" s="3">
+        <v>46218</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>252</v>
+      </c>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L25" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>254</v>
+      </c>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -2507,183 +2585,283 @@
         <v>30</v>
       </c>
       <c r="Q25" s="3"/>
-      <c r="R25" s="4" t="str">
+      <c r="R25" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="1:18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" hidden="1">
       <c r="A26" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
+      <c r="B26" s="3">
+        <v>46218</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>251</v>
+      </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L26" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="L26" s="2" t="s">
+        <v>255</v>
+      </c>
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
       <c r="O26" s="2"/>
       <c r="P26" s="2" t="s">
-        <v>30</v>
+        <v>186</v>
       </c>
       <c r="Q26" s="3"/>
-      <c r="R26" s="4" t="str">
+      <c r="R26" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="1:18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="28" hidden="1">
       <c r="A27" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="2"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
-      <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
+      <c r="B27" s="3">
+        <v>46218</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>256</v>
+      </c>
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L27" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="L27" s="2" t="s">
+        <v>255</v>
+      </c>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
       <c r="P27" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q27" s="3"/>
-      <c r="R27" s="4" t="str">
+        <v>186</v>
+      </c>
+      <c r="Q27" s="3">
+        <v>46218</v>
+      </c>
+      <c r="R27" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="1:18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="28" hidden="1">
       <c r="A28" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="3"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
+      <c r="B28" s="3">
+        <v>46218</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>256</v>
+      </c>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L28" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="L28" s="2" t="s">
+        <v>258</v>
+      </c>
       <c r="M28" s="2"/>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
       <c r="P28" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q28" s="3"/>
-      <c r="R28" s="4" t="str">
+        <v>186</v>
+      </c>
+      <c r="Q28" s="3">
+        <v>46218</v>
+      </c>
+      <c r="R28" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="1:18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" ht="28" hidden="1">
       <c r="A29" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B29" s="3"/>
-      <c r="C29" s="2"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-      <c r="F29" s="2"/>
-      <c r="G29" s="2"/>
+      <c r="B29" s="3">
+        <v>46218</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>262</v>
+      </c>
       <c r="H29" s="2"/>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L29" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="L29" s="2" t="s">
+        <v>259</v>
+      </c>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
-      <c r="O29" s="2"/>
+      <c r="O29" s="2" t="s">
+        <v>264</v>
+      </c>
       <c r="P29" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q29" s="3"/>
-      <c r="R29" s="4" t="str">
+        <v>186</v>
+      </c>
+      <c r="Q29" s="3">
+        <v>46218</v>
+      </c>
+      <c r="R29" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="1:18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" ht="28" hidden="1">
       <c r="A30" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B30" s="3"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
+      <c r="B30" s="3">
+        <v>46218</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>265</v>
+      </c>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
       <c r="K30" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L30" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>260</v>
+      </c>
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
       <c r="P30" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q30" s="3"/>
-      <c r="R30" s="4" t="str">
+        <v>186</v>
+      </c>
+      <c r="Q30" s="3">
+        <v>46218</v>
+      </c>
+      <c r="R30" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="1:18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" ht="28" hidden="1">
       <c r="A31" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
+      <c r="B31" s="3">
+        <v>46218</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>267</v>
+      </c>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
+      <c r="J31" s="2" t="s">
+        <v>270</v>
+      </c>
       <c r="K31" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L31" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="L31" s="2" t="s">
+        <v>261</v>
+      </c>
       <c r="M31" s="2"/>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2"/>
+      <c r="N31" t="s">
+        <v>269</v>
+      </c>
+      <c r="O31" s="2" t="s">
+        <v>271</v>
+      </c>
       <c r="P31" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q31" s="3"/>
-      <c r="R31" s="4" t="str">
+        <v>186</v>
+      </c>
+      <c r="Q31" s="3">
+        <v>46218</v>
+      </c>
+      <c r="R31" s="4">
         <f t="shared" ca="1" si="0"/>
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:18">
@@ -3387,7 +3565,7 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIF('Bug Tracker'!F2:F51,"&lt;&gt;")</f>
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C5" s="5"/>
       <c r="D5" s="5" t="s">
@@ -3395,7 +3573,7 @@
       </c>
       <c r="E5" s="5">
         <f>COUNTIF('Bug Tracker'!K2:K51,D5)</f>
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="F5" s="5"/>
       <c r="G5" s="5" t="s">
@@ -3403,7 +3581,7 @@
       </c>
       <c r="H5" s="5">
         <f>COUNTIF('Bug Tracker'!C2:C51,G5)</f>
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -3412,7 +3590,7 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIFS('Bug Tracker'!F2:F51,"&lt;&gt;",'Bug Tracker'!K2:K51,"&lt;&gt;Closed",'Bug Tracker'!K2:K51,"&lt;&gt;Verified")</f>
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
@@ -3428,7 +3606,7 @@
       </c>
       <c r="H6" s="5">
         <f>COUNTIF('Bug Tracker'!C2:C51,G6)</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -3437,7 +3615,7 @@
       </c>
       <c r="B7" s="5">
         <f>COUNTIF('Bug Tracker'!C2:C51,"Critical")</f>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C7" s="5"/>
       <c r="D7" s="5" t="s">
@@ -3462,7 +3640,7 @@
       </c>
       <c r="B8" s="5">
         <f>COUNTIF('Bug Tracker'!C2:C51,"High")</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C8" s="5"/>
       <c r="D8" s="5" t="s">
@@ -3478,7 +3656,7 @@
       </c>
       <c r="H8" s="5">
         <f>COUNTIF('Bug Tracker'!C2:C51,G8)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -3527,7 +3705,7 @@
       </c>
       <c r="B11" s="5">
         <f>COUNTIF('Bug Tracker'!K2:K51,"Closed")+COUNTIF('Bug Tracker'!K2:K51,"Verified")</f>
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="5" t="s">
@@ -3565,7 +3743,7 @@
       </c>
       <c r="E13" s="5">
         <f>COUNTIF('Bug Tracker'!K2:K51,D13)</f>
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>

</xml_diff>